<commit_message>
docs: plan de pruebas 1.1 (86 casos) y guía 1.2 con lo de la reunión del 21-10
- Plan de pruebas: 21 casos nuevos (retiros y gastos, tutorial, alta de
  negocios y límites, logo/color/suspender, privacidad del soporte) y C09
  con montos concretos para el arreglo de abonos. Instrucciones en tuteo.
- Guía 1.2: tutorial y "Ver tutorial", "Acceso suspendido", alta de
  negocios y límites por plan, suspender y último acceso, 4.5 Tu
  privacidad y el soporte, primeros pasos, logo y color, retiros y gastos
  en Cierre y en Finanzas, matriz de permisos y preguntas frecuentes.
  Matriz compactada para que entre con su título. PDF de 24 páginas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/plan-de-pruebas-farmacia.xlsx
+++ b/docs/qa/plan-de-pruebas-farmacia.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuario nuevo" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Transversal'!$A$1:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Admin'!$A$1:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dueño'!$A$1:$H$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Regente'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cajero'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Transversal'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Admin'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dueño'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Regente'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cajero'!$A$1:$H$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Usuario nuevo'!$A$1:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.0 · octubre de 2026</t>
+          <t>Versión 1.1 · 21 de octubre de 2026</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Cada hoja es un rol. Por caso: hacé los pasos, compará con 'Resultado esperado' y marcá Pasó = Sí o No. Si es No, escribí qué pasó (mensaje exacto, pantalla, hora) y, si podés, una captura con el ID del caso en el nombre del archivo. Quién probó y Fecha ayudan a reproducir.</t>
+          <t>Cada hoja es un rol. Por caso: haz los pasos, compara con 'Resultado esperado' y marca Pasó = Sí o No. Si es No, escribe qué pasó (mensaje exacto, pantalla, hora) y, si puedes, agrega una captura con el ID del caso en el nombre del archivo. Quién probó y Fecha ayudan a reproducir.</t>
         </is>
       </c>
     </row>
@@ -567,14 +567,14 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Orden sugerido</t>
+          <t>Novedades de la versión 1.1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>1) Transversal T01–T07 · 2) Admin · 3) Dueño (deja los datos de prueba del D01 creados) · 4) Regente · 5) Cajero · 6) Usuario nuevo · 7) Transversal T08–T13.</t>
+          <t>Lo de la reunión del 21 de octubre: retiros y gastos de caja (C14, C15, R13, R14, D15, D16), tutorial (T14, C16, C17), alta de negocios y límites por plan (A10–A13, D20, D21), logo, color y suspender (D17, D18, D22) y privacidad del soporte (A14, A15, D19). C09 ahora prueba el cobro de encargos con montos concretos. Estos casos requieren que estén desplegados los cambios correspondientes y corridos sus SQL.</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,29 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Qué NO cubre este plan</t>
+          <t>Orden sugerido</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>1) Transversal T01–T07 · 2) Admin · 3) Dueño (deja los datos de prueba del D01 creados) · 4) Regente · 5) Cajero · 6) Usuario nuevo · 7) Transversal T08–T13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Qué NO cubre este plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Boleta electrónica (el POS emite un comprobante interno, no documento tributario), respaldos y cargas masivas: se prueban aparte.</t>
         </is>
@@ -601,722 +618,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Pantalla</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Pasos</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Resultado esperado</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Pasó</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Observación / falla</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Quién probó</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>T01</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Entrar con una cuenta de QA y su contraseña.</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Abre 'Mis portales' con la tarjeta Farmacia.</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>T02</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Entrar con una contraseña incorrecta.</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Mensaje 'Correo o contraseña incorrectos'. No entra.</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>T03</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Olvidé mi contraseña</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Pedir el enlace para QA Cajero (su correo llega a la bandeja del superadmin). Abrirlo y definir una contraseña nueva.</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Llega el correo; el enlace abre la pantalla de nueva contraseña; con la nueva se entra.</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>T04</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Cambiar contraseña</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Menú de cuenta → Cambiar contraseña. Primero con la actual mal escrita; después bien.</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Con la actual incorrecta: error. Con la correcta: 'Contraseña actualizada' y se entra con la nueva.</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>T05</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Barra del portal</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Dentro de Farmacia, usar 'Cerrar sesión' de la barra. Luego botón Atrás del navegador.</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Vuelve a /login. Atrás no muestra pantallas con datos.</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Barra del portal</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Dentro de Farmacia, usar 'Mis portales'. Como admin, 'Panel admin'.</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Los botones están siempre visibles a la derecha, aunque la barra de secciones tenga scroll.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Moneda</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Recorrer POS, Ventas, Inventario y Finanzas en la Farmacia de Prueba (CLP).</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Todos los montos salen como $ 9.530 (punto de miles, sin decimales). Fechas en formato chileno.</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>T08</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Registro</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Con QA Nuevo: 'Crear una cuenta' en /signup, confirmar el correo, iniciar sesión.</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Llega el correo de confirmación; al entrar muestra 'Aprobación pendiente'.</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>T09</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Alta por el dueño</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Como dueño: Equipo → Agregar persona → 'Ya tiene cuenta' con el correo de QA Nuevo, rol cajero. Luego entrar con QA Nuevo.</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Queda en el equipo al instante; QA Nuevo entra directo a Farmacia sin esperar aprobación.</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>T10</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Contraseña inicial</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Entrar con una cuenta creada desde Equipo ('Crear cuenta nueva'). Intentar ir a /portal/farmacia escribiendo la URL.</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Siempre redirige a 'Elige tu contraseña' hasta que la cambie.</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>T11</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Contraseña inicial</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>En esa pantalla, poner la inicial y elegir una nueva.</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Entra a Mis portales; en los siguientes ingresos ya no la pide.</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>T12</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Admin en 'ver como'</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Como superadmin (o QA Admin): Usuarios → ⋯ → 'Ver sus portales' del dueño de prueba → Farmacia → POS.</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Entra en solo lectura: la barra azul avisa; 'Cobrar' deshabilitado; crear producto no aparece. 'Volver a mi cuenta' sale del modo.</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>T13</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Cambio de cuenta</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Cerrar sesión estando en 'ver como' y entrar como QA Cajero en el mismo navegador. Hacer una venta.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>La venta se registra (no aparece 'modo lectura').</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H14"/>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No,Parcial"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Pantalla</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Pasos</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Resultado esperado</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Pasó</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Observación / falla</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Quién probó</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Panel admin · inicio</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Entrar como QA Admin.</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Tarjeta 'Mantenimiento diario' en verde con la última ejecución de hoy. Botón 'Ejecutar ahora' funciona y actualiza la hora.</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Usuarios · Crear usuario</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Crear un usuario con contraseña generada. Repetir como QA Superadmin.</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>QA Admin no ve la opción 'Administrador'; QA Superadmin sí. Las credenciales se muestran una sola vez y se copian.</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>A03</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Usuarios · Crear usuario</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Intentar crear con un correo ya existente.</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Mensaje claro: ya existe una cuenta con ese correo.</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>A04</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Usuarios</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Aprobar a QA Nuevo (si sigue pendiente), suspenderlo, reactivarlo. Entre cada paso, intentar entrar con QA Nuevo.</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente → 'Aprobación pendiente'; suspendido → 'Cuenta suspendida'; reactivado → entra.</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>A05</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Usuarios · Membresía</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Asignar y extender la membresía del dueño de prueba.</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>La fecha de vencimiento cambia; el dueño y su equipo entran al portal.</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>A06</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Usuarios · Acceso a portales</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Quitar y volver a dar acceso a Farmacia al dueño de prueba.</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Sin acceso: 'Sin acceso a este portal'. Con acceso: entra.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>A07</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Usuarios · Cambiar rol</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Como QA Admin, buscar la opción de cambiar rol.</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>No aparece (solo superadmin).</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>A08</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Auditoría</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Después de A02–A06, abrir Admin → Auditoría.</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Aparecen las acciones con quién, cuándo y sobre quién.</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>A09</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Alertas</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Admin → Alertas con una membresía que venza en menos de 7 días.</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>La membresía figura en la lista de próximas a vencer.</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H10"/>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No,Parcial"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1380,22 +681,22 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Inicio · Alertas de hoy</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Preparar en la Farmacia de Prueba: un lote vencido con stock, uno que vence en 30 días, uno sin fecha, un producto con mínimo 10 y 4 unidades, un tratamiento crónico a 1 día, una cuenta por pagar vencida. Abrir el inicio.</t>
+          <t>Entrar con una cuenta de QA y su contraseña.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>6 tarjetas con los conteos correctos. Cada una abre la pantalla con el filtro aplicado y el mismo número de filas.</t>
+          <t>Abre 'Mis portales' con la tarjeta Farmacia.</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr"/>
@@ -1406,22 +707,22 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Inicio · Alertas de hoy</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Corregir la fecha del lote vencido y volver al inicio.</t>
+          <t>Entrar con una contraseña incorrecta.</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>La tarjeta de vencidos desaparece al instante. Sin datos de prueba: 'Todo en orden'.</t>
+          <t>Mensaje 'Correo o contraseña incorrectos'. No entra.</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr"/>
@@ -1432,22 +733,22 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Inicio · Datos del negocio</t>
+          <t>Olvidé mi contraseña</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Botón 'Datos del negocio': cambiar nombre, RUT, dirección y teléfono.</t>
+          <t>Pedir el enlace para QA Cajero (su correo llega a la bandeja del superadmin). Abrirlo y definir una contraseña nueva.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>La etiqueta dice RUT (farmacia chilena). Al guardar, cambia el nombre en la cabecera y la línea gris bajo el nombre.</t>
+          <t>Llega el correo; el enlace abre la pantalla de nueva contraseña; con la nueva se entra.</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr"/>
@@ -1458,22 +759,22 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Equipo · Crear cuenta nueva</t>
+          <t>Cambiar contraseña</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Agregar persona → 'Crear cuenta nueva' con nombre, correo (+qa-cajero2 del Gmail), rol cajero, contraseña generada.</t>
+          <t>Menú de cuenta → Cambiar contraseña. Primero con la actual mal escrita; después bien.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Queda en el equipo con el rol elegido. Se muestran usuario y contraseña una sola vez con botón Copiar.</t>
+          <t>Con la actual incorrecta: error. Con la correcta: 'Contraseña actualizada' y se entra con la nueva.</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
@@ -1484,22 +785,22 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Barra del portal</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Cambiar el rol de QA Cajero a regente y volver a cajero. Quitar a QA Nuevo del equipo.</t>
+          <t>Dentro de Farmacia, usar 'Cerrar sesión' de la barra. Luego botón Atrás del navegador.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Los cambios se ven al instante; QA Nuevo pierde el acceso al portal.</t>
+          <t>Vuelve a /login. Atrás no muestra pantallas con datos.</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
@@ -1510,22 +811,22 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Equipo · Auditoría de accesos</t>
+          <t>Barra del portal</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Mirar la sección de accesos.</t>
+          <t>Dentro de Farmacia, usar 'Mis portales'. Como admin, 'Panel admin'.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Aparecen los inicios y cierres de sesión recientes de cada miembro.</t>
+          <t>Los botones están siempre visibles a la derecha, aunque la barra de secciones tenga scroll.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
@@ -1536,22 +837,22 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Nuevo producto</t>
+          <t>Moneda</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Crear un producto con precio 10.000, costo neto 5.000, IVA 19, stock mínimo 5.</t>
+          <t>Recorrer POS, Ventas, Inventario y Finanzas en la Farmacia de Prueba (CLP).</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>El formulario muestra costo con IVA 5.950, utilidad 4.050 y margen 41 % antes de guardar. En la tabla: Costo c/IVA y Margen.</t>
+          <t>Todos los montos salen como $ 9.530 (punto de miles, sin decimales). Fechas en formato chileno.</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
@@ -1562,22 +863,22 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Editar</t>
+          <t>Registro</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Editar el precio desde el lápiz de la fila y desde 'Editar producto' en el detalle.</t>
+          <t>Con QA Nuevo: 'Crear una cuenta' en /signup, confirmar el correo, iniciar sesión.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>El cambio se refleja; en el detalle, 'Historial de cambios' muestra precio anterior → nuevo, con quién y cuándo.</t>
+          <t>Llega el correo de confirmación; al entrar muestra 'Aprobación pendiente'.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr"/>
@@ -1588,22 +889,22 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Eliminar</t>
+          <t>Alta por el dueño</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Eliminar un producto de prueba.</t>
+          <t>Como dueño: Equipo → Agregar persona → 'Ya tiene cuenta' con el correo de QA Nuevo, rol cajero. Luego entrar con QA Nuevo.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Desaparece de la tabla; queda en la auditoría.</t>
+          <t>Queda en el equipo al instante; QA Nuevo entra directo a Farmacia sin esperar aprobación.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
@@ -1614,22 +915,22 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>Contraseña inicial</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Abrir Finanzas.</t>
+          <t>Entrar con una cuenta creada desde Equipo ('Crear cuenta nueva'). Intentar ir a /portal/farmacia escribiendo la URL.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>KPIs del mes, ingresos por método, últimos cierres, 'Inventario valorizado' (a costo, a venta, unidades, por categoría) y 'Día a día'. Los CSV abren en Excel con tildes correctas.</t>
+          <t>Siempre redirige a 'Elige tu contraseña' hasta que la cambie.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr"/>
@@ -1640,22 +941,22 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Finanzas · Valorización</t>
+          <t>Contraseña inicial</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Elegir 3 productos con stock, calcular a mano unidades × costo con IVA y comparar con el CSV.</t>
+          <t>En esa pantalla, poner la inicial y elegir una nueva.</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Coinciden.</t>
+          <t>Entra a Mis portales; en los siguientes ingresos ya no la pide.</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
@@ -1666,22 +967,22 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Admin en 'ver como'</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Crear una cuenta por pagar, abonarla parcialmente, anularla.</t>
+          <t>Como superadmin (o QA Admin): Usuarios → ⋯ → 'Ver sus portales' del dueño de prueba → Farmacia → POS.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Estados pendiente → parcial → anulada. Solo el dueño ve 'Anular'.</t>
+          <t>Entra en solo lectura: la barra azul avisa; 'Cobrar' deshabilitado; crear producto no aparece. 'Volver a mi cuenta' sale del modo.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr"/>
@@ -1692,22 +993,22 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Cierre</t>
+          <t>Cambio de cuenta</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Abrir Cierre como dueño.</t>
+          <t>Cerrar sesión estando en 'ver como' y entrar como QA Cajero en el mismo navegador. Hacer una venta.</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Ve los totales esperados por método y los movimientos del turno (el cajero no).</t>
+          <t>La venta se registra (no aparece 'modo lectura').</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr"/>
@@ -1718,22 +1019,22 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Mostrar más</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Con los 665 productos cargados, abrir Inventario y escribir rápido en el buscador.</t>
+          <t>Con cualquier cuenta del portal: 'Ver tutorial' en la barra. Recorrerlo con Siguiente/Anterior y probar 'Ir ahora' en un paso.</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>No se traba. Si hay más de 200 resultados aparece 'Mostrar 200 más'; los contadores de la barra no cambian.</t>
+          <t>Se abre desde el paso 1, muestra 'Paso N de M' y 'Ir ahora' lleva a la pantalla del paso.</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr"/>
@@ -1752,13 +1053,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1816,22 +1117,22 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>Panel admin · inicio</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Entrar como QA Regente a Finanzas.</t>
+          <t>Entrar como QA Admin.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Pantalla bloqueada: 'exclusiva del dueño'.</t>
+          <t>Tarjeta 'Mantenimiento diario' en verde con la última ejecución de hoy. Botón 'Ejecutar ahora' funciona y actualiza la hora.</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr"/>
@@ -1842,22 +1143,22 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Inicio / Equipo</t>
+          <t>Usuarios · Crear usuario</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Buscar el botón 'Datos del negocio' y 'Agregar persona'.</t>
+          <t>Crear un usuario con contraseña generada. Repetir como QA Superadmin.</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>No aparecen (solo dueño). Sí ve la auditoría de accesos.</t>
+          <t>QA Admin no ve la opción 'Administrador'; QA Superadmin sí. Las credenciales se muestran una sola vez y se copian.</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr"/>
@@ -1868,22 +1169,22 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>R03</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Lotes</t>
+          <t>Usuarios · Crear usuario</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>En un producto: ingresar un lote con fecha y otro sin fecha.</t>
+          <t>Intentar crear con un correo ya existente.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>El sin fecha queda gris 'Sin fecha' con botón 'Completar fecha'.</t>
+          <t>Mensaje claro: ya existe una cuenta con ese correo.</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr"/>
@@ -1894,22 +1195,22 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Editar lote</t>
+          <t>Usuarios</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Completar la fecha del lote sin fecha. Luego intentar borrarle la fecha a un lote que la tiene.</t>
+          <t>Aprobar a QA Nuevo (si sigue pendiente), suspenderlo, reactivarlo. Entre cada paso, intentar entrar con QA Nuevo.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>La primera se guarda y el semáforo cambia. La segunda se rechaza: 'no puede quedar sin fecha'.</t>
+          <t>Pendiente → 'Aprobación pendiente'; suspendido → 'Cuenta suspendida'; reactivado → entra.</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
@@ -1920,22 +1221,22 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>R05</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Movimientos</t>
+          <t>Usuarios · Membresía</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Pasar unidades de bodega a venta, registrar una merma con motivo.</t>
+          <t>Asignar y extender la membresía del dueño de prueba.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Las cantidades cambian; ambos quedan en 'Movimientos recientes' con el motivo.</t>
+          <t>La fecha de vencimiento cambia; el dueño y su equipo entran al portal.</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
@@ -1946,22 +1247,22 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>R06</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Filtros</t>
+          <t>Usuarios · Acceso a portales</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Usar Vencidos, Por vencer, Sin fecha, Bajo mínimo, Sin stock, Inactivos. Probar la URL ?filtro=bajo_minimo y ?filtro=loquesea.</t>
+          <t>Quitar y volver a dar acceso a Farmacia al dueño de prueba.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Cada filtro muestra solo lo que corresponde; la URL abre con el filtro; un valor inválido cae en 'Todos'.</t>
+          <t>Sin acceso: 'Sin acceso a este portal'. Con acceso: entra.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
@@ -1972,22 +1273,22 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>R07</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Stock mínimo</t>
+          <t>Usuarios · Cambiar rol</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Poner mínimo 10 a un producto con 4 unidades.</t>
+          <t>Como QA Admin, buscar la opción de cambiar rol.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Chip 'Bajo mínimo' en la fila, píldora en la barra y tarjeta en el inicio. Con mínimo 2 desaparecen.</t>
+          <t>No aparece (solo superadmin).</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
@@ -1998,22 +1299,22 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>R08</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Ventas · Anular</t>
+          <t>Auditoría</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Anular una venta con motivo.</t>
+          <t>Después de A02–A06, abrir Admin → Auditoría.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Queda marcada ANULADA con el motivo; el stock vuelve al lote del que salió.</t>
+          <t>Aparecen las acciones con quién, cuándo y sobre quién.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr"/>
@@ -2024,22 +1325,22 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>R09</t>
+          <t>A09</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Pedidos</t>
+          <t>Alertas</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Cancelar un pedido con motivo.</t>
+          <t>Admin → Alertas con una membresía que venza en menos de 7 días.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Queda cancelado; si tenía anticipo, aparece el aviso de devolverlo.</t>
+          <t>La membresía figura en la lista de próximas a vencer.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
@@ -2050,22 +1351,22 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Planes · Límites</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Crear y abonar una cuenta por pagar; buscar 'Anular'.</t>
+          <t>Admin → Planes: editar un plan y poner Máx. regentes 1 y Máx. cajeros 2. Dejar otro plan con los campos vacíos.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Crear y abonar funcionan; 'Anular' no aparece.</t>
+          <t>La tarjeta del plan muestra '1 regente · 2 cajeros'; el vacío dice 'sin límite'.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr"/>
@@ -2076,22 +1377,22 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>A11</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Inventario · Costos</t>
+          <t>Negocios · Nuevo negocio</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Mirar la tabla y el detalle.</t>
+          <t>Admin → Negocios → Nuevo negocio: 'Farmacia QA Alta', Chile, dueño nuevo (+qa-dueno2 del Gmail), plan con límites, 1 cajero (+qa-cajero3). Dar de alta.</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Ve Costo c/IVA, Margen y el historial de cambios.</t>
+          <t>Muestra las dos contraseñas iniciales una sola vez. La lista suma el negocio con su plan, vencimiento y '1 de 2' cajeros.</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
@@ -2102,22 +1403,22 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Lotes sin fecha en el POS</t>
+          <t>Negocios · Dueño del alta</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Producto con un lote con fecha y otro sin fecha: venderlo.</t>
+          <t>Entrar con el dueño recién creado.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Se descuenta primero el lote con fecha (FEFO); el sin fecha va al final.</t>
+          <t>Pide elegir contraseña; el portal sale en CLP; al crear un producto propone IVA 19; Equipo muestra al cajero.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr"/>
@@ -2125,10 +1426,88 @@
       <c r="G13" s="7" t="inlineStr"/>
       <c r="H13" s="7" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>A13</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Negocios · Todo o nada</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Repetir el alta usando como dueño 'Ya tiene cuenta' con el correo del dueño de la Farmacia de Prueba.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Error 'Esa cuenta ya pertenece a otro negocio… Se deshizo lo que se había creado'. En Usuarios no quedó ninguna cuenta nueva.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Ver como · Privacidad</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>En 'ver como' del dueño de prueba (sin permiso de soporte): abrir Ventas, Finanzas, Recetas, Inventario y Equipo.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Ventas, Finanzas y Recetas muestran 'sin permiso de soporte'. Inventario y Equipo se ven. El inicio avisa que pacientes y cuentas aparecen en cero.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Ver como · Con permiso</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Después del D19 (el dueño da permiso), recargar Ventas en 'ver como'. Luego el dueño quita el permiso y recargar otra vez.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Con permiso se ven las ventas (sin poder cobrar ni anular). Sin permiso vuelve el aviso. En Auditoría figuran 'autorizar_soporte' y 'revocar_soporte'.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H16"/>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No,Parcial"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2136,13 +1515,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2200,22 +1579,22 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>POS · Buscar</t>
+          <t>Inicio · Alertas de hoy</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Escribir o escanear un código de barras y Enter. Escribir 'acido' sin tilde.</t>
+          <t>Preparar en la Farmacia de Prueba: un lote vencido con stock, uno que vence en 30 días, uno sin fecha, un producto con mínimo 10 y 4 unidades, un tratamiento crónico a 1 día, una cuenta por pagar vencida. Abrir el inicio.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>El producto entra al ticket al instante. 'acido' encuentra los 'Ácido…'.</t>
+          <t>6 tarjetas con los conteos correctos. Cada una abre la pantalla con el filtro aplicado y el mismo número de filas.</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr"/>
@@ -2226,22 +1605,22 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>POS · Sin stock</t>
+          <t>Inicio · Alertas de hoy</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Buscar un producto con stock 0 que tenga principio activo.</t>
+          <t>Corregir la fecha del lote vencido y volver al inicio.</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Aparece deshabilitado con 'Equivalentes con stock' debajo, si hay otros con el mismo principio activo.</t>
+          <t>La tarjeta de vencidos desaparece al instante. Sin datos de prueba: 'Todo en orden'.</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr"/>
@@ -2252,22 +1631,22 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>POS · Pago mixto</t>
+          <t>Inicio · Datos del negocio</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Vender $ 10.000 pagando $ 6.000 débito + $ 5.000 efectivo.</t>
+          <t>Botón 'Datos del negocio': cambiar nombre, RUT, dirección y teléfono.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Vuelto $ 1.000 (sale del efectivo). Si lo electrónico supera el total, el botón se bloquea con aviso.</t>
+          <t>La etiqueta dice RUT (farmacia chilena). Al guardar, cambia el nombre en la cabecera y la línea gris bajo el nombre.</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr"/>
@@ -2278,22 +1657,22 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>POS · Receta</t>
+          <t>Equipo · Crear cuenta nueva</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Vender un producto Rx.</t>
+          <t>Agregar persona → 'Crear cuenta nueva' con nombre, correo (+qa-cajero2 del Gmail), rol cajero, contraseña generada.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Pide paciente, documento, médico y número de receta; sin eso no deja cobrar. Luego aparece en Recetas.</t>
+          <t>Queda en el equipo con el rol elegido. Se muestran usuario y contraseña una sola vez con botón Copiar.</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
@@ -2304,22 +1683,22 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>POS · Cliente</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Toca 'Cliente': escribir 1 letra, luego 2; crear un cliente nuevo y usarlo.</t>
+          <t>Cambiar el rol de QA Cajero a regente y volver a cajero. Quitar a QA Nuevo del equipo.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Con 1 letra pide 2; con 2 muestra resultados; el nuevo queda seleccionado sin recargar la página.</t>
+          <t>Los cambios se ven al instante; QA Nuevo pierde el acceso al portal.</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
@@ -2330,22 +1709,22 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>POS · Después de vender</t>
+          <t>Equipo · Auditoría de accesos</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Vender 2 unidades de un producto y mirar su stock en la lista. Tocar 'Imprimir' en el aviso verde.</t>
+          <t>Mirar la sección de accesos.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>El stock baja al instante sin recarga. Se abre el comprobante; al imprimir (o 'Guardar como PDF') sale solo el ticket.</t>
+          <t>Aparecen los inicios y cierres de sesión recientes de cada miembro.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
@@ -2356,22 +1735,22 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>POS · Dos cajeros</t>
+          <t>Inventario · Nuevo producto</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>En dos navegadores, con QA Cajero y el dueño, agregar la última unidad del mismo producto y cobrar en ambos.</t>
+          <t>Crear un producto con precio 10.000, costo neto 5.000, IVA 19, stock mínimo 5.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>El segundo recibe 'Stock insuficiente' o 'El stock cambió'; su ticket se corrige solo.</t>
+          <t>El formulario muestra costo con IVA 5.950, utilidad 4.050 y margen 41 % antes de guardar. En la tabla: Costo c/IVA y Margen.</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
@@ -2382,22 +1761,22 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Inventario · Editar</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Abrir Ventas; usar 'Hoy', '7 días', un rango manual; exportar CSV; reimprimir una venta con la impresora.</t>
+          <t>Editar el precio desde el lápiz de la fila y desde 'Editar producto' en el detalle.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>La lista y los KPIs cambian con el rango; el CSV abre en Excel; el comprobante se ve igual al del POS. No aparece el botón de anular.</t>
+          <t>El cambio se refleja; en el detalle, 'Historial de cambios' muestra precio anterior → nuevo, con quién y cuándo.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr"/>
@@ -2408,22 +1787,22 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Pedidos</t>
+          <t>Inventario · Eliminar</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Crear un encargo con anticipo, avanzarlo de estado y entregarlo cobrando el saldo.</t>
+          <t>Eliminar un producto de prueba.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>El saldo se cobra al entregar y el pago aparece en Ventas → Encargos.</t>
+          <t>Desaparece de la tabla; queda en la auditoría.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
@@ -2434,22 +1813,22 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Pacientes</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Crear un tratamiento (30 días), renovarlo, desactivarlo.</t>
+          <t>Abrir Finanzas.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Aparece en la lista con 'Se le acaba'; renovar actualiza la fecha; desactivado queda 'Pausado'.</t>
+          <t>KPIs del mes, ingresos por método, últimos cierres, 'Inventario valorizado' (a costo, a venta, unidades, por categoría) y 'Día a día'. Los CSV abren en Excel con tildes correctas.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr"/>
@@ -2460,22 +1839,22 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Cierre de caja</t>
+          <t>Finanzas · Valorización</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Cerrar caja declarando lo contado por método.</t>
+          <t>Elegir 3 productos con stock, calcular a mano unidades × costo con IVA y comparar con el CSV.</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>No se ve el total esperado antes de declarar. Después muestra la diferencia. A los 30 s cierra la sesión (o con 'Salir ahora').</t>
+          <t>Coinciden.</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
@@ -2486,22 +1865,22 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Permisos</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Recorrer Inventario, Finanzas, Compras y Equipo.</t>
+          <t>Crear una cuenta por pagar, abonarla parcialmente, anularla.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Inventario sin Costo/Margen ni lápiz de editar; Finanzas y Compras bloqueadas; Equipo solo lectura.</t>
+          <t>Estados pendiente → parcial → anulada. Solo el dueño ve 'Anular'.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr"/>
@@ -2512,22 +1891,22 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>POS en tablet</t>
+          <t>Cierre</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Abrir el POS en una tablet o con el navegador a 800 px de ancho.</t>
+          <t>Abrir Cierre como dueño.</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Buscador, resultados y ticket usables sin scroll horizontal.</t>
+          <t>Ve los totales esperados por método y los movimientos del turno (el cajero no).</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr"/>
@@ -2535,10 +1914,1194 @@
       <c r="G14" s="7" t="inlineStr"/>
       <c r="H14" s="7" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Mostrar más</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Con los 665 productos cargados, abrir Inventario y escribir rápido en el buscador.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>No se traba. Si hay más de 200 resultados aparece 'Mostrar 200 más'; los contadores de la barra no cambian.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Cierre · Retiros y gastos</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Después del C14, abrir Cierre como dueño.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Los totales del turno muestran 'Retiros: −$ 50.000' y 'Gastos: −$ 5.000'; los movimientos aparecen con signo menos y quién los hizo.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Finanzas · Gastos del mes</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Abrir Finanzas y exportar el CSV de 'Gastos y retiros de caja del mes'.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Gastos por categoría (Insumos $ 5.000) y retiros aparte, con la nota 'no es gasto'. El CSV trae fecha, tipo, categoría, concepto y monto.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Datos del negocio · Logo y color</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Subir un logo PNG chico, elegir el color Verde. Después intentar subir un SVG y una imagen de más de 500 KB.</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>El logo sale en la barra, el inicio y el comprobante; la pestaña activa queda verde. El SVG y la imagen grande se rechazan con mensaje.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Equipo · Suspender</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Con QA Cajero con la sesión abierta en otro navegador: suspenderlo desde ⋯. Que QA Cajero haga clic en cualquier sección. Luego reactivarlo.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>La tarjeta queda 'Suspendido'. QA Cajero sale a Mis portales con 'Acceso suspendido'. Al reactivarlo, vuelve a entrar.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Inicio · Soporte de LOMS 360</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>En la tarjeta 'Soporte de LOMS 360': 'Permitir por 24 h'. Después 'Quitar permiso'.</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Muestra 'hasta [fecha y hora]' mientras está activo; al quitarlo vuelve a 'tus datos son privados'.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr"/>
+      <c r="F20" s="7" t="inlineStr"/>
+      <c r="G20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Inicio · Primeros pasos</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>En un negocio nuevo (el del A11), entrar como dueño y completar cada paso.</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>La lista marca cada paso al cumplirse y desaparece cuando están todos.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="7" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Equipo · Cupo del plan</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>En el negocio del A11 (plan con 2 cajeros): agregar un segundo cajero, luego intentar un tercero y cambiar a alguien a cajero.</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Arriba dice '2 de 2 cajeros'; el rol Cajero queda deshabilitado con 'Tu plan no permite más personas con este rol' y en el menú dice '(cupo lleno)'.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Equipo · Último acceso</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Mirar las tarjetas del equipo.</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Cada persona muestra 'Último acceso' y, salvo el dueño, 'último cierre' (o 'nunca' / 'ninguno').</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="7" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr"/>
+      <c r="H23" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H23"/>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No,Parcial"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Pantalla</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Pasos</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Resultado esperado</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Pasó</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Observación / falla</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Quién probó</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Finanzas</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Entrar como QA Regente a Finanzas.</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Pantalla bloqueada: 'exclusiva del dueño'.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr"/>
+      <c r="F2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>R02</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Inicio / Equipo</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Buscar el botón 'Datos del negocio' y 'Agregar persona'.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>No aparecen (solo dueño). Sí ve la auditoría de accesos.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>R03</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Lotes</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>En un producto: ingresar un lote con fecha y otro sin fecha.</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>El sin fecha queda gris 'Sin fecha' con botón 'Completar fecha'.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>R04</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Editar lote</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Completar la fecha del lote sin fecha. Luego intentar borrarle la fecha a un lote que la tiene.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>La primera se guarda y el semáforo cambia. La segunda se rechaza: 'no puede quedar sin fecha'.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Movimientos</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Pasar unidades de bodega a venta, registrar una merma con motivo.</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Las cantidades cambian; ambos quedan en 'Movimientos recientes' con el motivo.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Filtros</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Usar Vencidos, Por vencer, Sin fecha, Bajo mínimo, Sin stock, Inactivos. Probar la URL ?filtro=bajo_minimo y ?filtro=loquesea.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Cada filtro muestra solo lo que corresponde; la URL abre con el filtro; un valor inválido cae en 'Todos'.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Stock mínimo</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Poner mínimo 10 a un producto con 4 unidades.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Chip 'Bajo mínimo' en la fila, píldora en la barra y tarjeta en el inicio. Con mínimo 2 desaparecen.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Ventas · Anular</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Anular una venta con motivo.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Queda marcada ANULADA con el motivo; el stock vuelve al lote del que salió.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>R09</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Cancelar un pedido con motivo.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Queda cancelado; si tenía anticipo, aparece el aviso de devolverlo.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Crear y abonar una cuenta por pagar; buscar 'Anular'.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Crear y abonar funcionan; 'Anular' no aparece.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Inventario · Costos</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Mirar la tabla y el detalle.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Ve Costo c/IVA, Margen y el historial de cambios.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Lotes sin fecha en el POS</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Producto con un lote con fecha y otro sin fecha: venderlo.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Se descuenta primero el lote con fecha (FEFO); el sin fecha va al final.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Cierre · Anular un gasto</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Anular con motivo un gasto registrado por QA Cajero en el turno abierto (la X de la fila). Cerrar caja.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>El gasto queda tachado 'anulado: motivo' y el cierre no lo descuenta.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Cierre · Turno cerrado</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Intentar anular un retiro de un turno que ya se cerró (por ejemplo, desde otra pestaña abierta antes del cierre).</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Se rechaza: 'ya entró en un cierre de caja'.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H15"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No,Parcial"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Pantalla</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Pasos</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Resultado esperado</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Pasó</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Observación / falla</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Quién probó</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>POS · Buscar</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Escribir o escanear un código de barras y Enter. Escribir 'acido' sin tilde.</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>El producto entra al ticket al instante. 'acido' encuentra los 'Ácido…'.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr"/>
+      <c r="F2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>POS · Sin stock</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Buscar un producto con stock 0 que tenga principio activo.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Aparece deshabilitado con 'Equivalentes con stock' debajo, si hay otros con el mismo principio activo.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>POS · Pago mixto</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Vender $ 10.000 pagando $ 6.000 débito + $ 5.000 efectivo.</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Vuelto $ 1.000 (sale del efectivo). Si lo electrónico supera el total, el botón se bloquea con aviso.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>POS · Receta</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Vender un producto Rx.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Pide paciente, documento, médico y número de receta; sin eso no deja cobrar. Luego aparece en Recetas.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>POS · Cliente</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Toca 'Cliente': escribir 1 letra, luego 2; crear un cliente nuevo y usarlo.</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Con 1 letra pide 2; con 2 muestra resultados; el nuevo queda seleccionado sin recargar la página.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>POS · Después de vender</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Vender 2 unidades de un producto y mirar su stock en la lista. Tocar 'Imprimir' en el aviso verde.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>El stock baja al instante sin recarga. Se abre el comprobante; al imprimir (o 'Guardar como PDF') sale solo el ticket.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>POS · Dos cajeros</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>En dos navegadores, con QA Cajero y el dueño, agregar la última unidad del mismo producto y cobrar en ambos.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>El segundo recibe 'Stock insuficiente' o 'El stock cambió'; su ticket se corrige solo.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Abrir Ventas; usar 'Hoy', '7 días', un rango manual; exportar CSV; reimprimir una venta con la impresora.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>La lista y los KPIs cambian con el rango; el CSV abre en Excel; el comprobante se ve igual al del POS. No aparece el botón de anular.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Crear un encargo de $ 10.000 con anticipo de $ 4.000 en efectivo, avanzarlo hasta 'recibido' y usar 'Entregar y cobrar' pagando los $ 6.000 con débito.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>La entrega pasa sin error. En Ventas → Encargos aparecen los dos pagos. En el cierre del turno, lo esperado suma $ 4.000 en efectivo y $ 6.000 en débito.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Pacientes</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Crear un tratamiento (30 días), renovarlo, desactivarlo.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Aparece en la lista con 'Se le acaba'; renovar actualiza la fecha; desactivado queda 'Pausado'.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Cierre de caja</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Cerrar caja declarando lo contado por método.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>No se ve el total esperado antes de declarar. Después muestra la diferencia. A los 30 s cierra la sesión (o con 'Salir ahora').</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Permisos</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Recorrer Inventario, Finanzas, Compras y Equipo.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Inventario sin Costo/Margen ni lápiz de editar; Finanzas y Compras bloqueadas; Equipo solo lectura.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>POS en tablet</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Abrir el POS en una tablet o con el navegador a 800 px de ancho.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Buscador, resultados y ticket usables sin scroll horizontal.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Cierre · Retiro y gasto</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>En un turno con una venta de $ 60.000 en efectivo: 'Retiro de caja' de $ 50.000 ('remesa para el dueño') y 'Gasto' de $ 5.000 ('bidón de agua', Insumos). Cerrar declarando $ 5.000 en efectivo.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Los dos aparecen en Movimientos del turno con signo menos. El cierre da diferencia 0 y dice que ya descuenta los retiros y gastos.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Cierre · Anular lo propio</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Registrar un gasto con un monto mal escrito y anularlo con la X, indicando el motivo.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Queda tachado con 'anulado: motivo'. No aparece la X en movimientos de otras personas.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Tutorial · Primer ingreso</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Entrar con una cuenta de cajero nueva (creada en D04), elegir contraseña.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Se abre solo el tutorial de cajero: vender, cobrar, recetas, encargos, retiros y gastos, cierre. No menciona Finanzas ni Equipo.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Tutorial · No se repite</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Tocar 'Saltar tutorial', recargar la página, cerrar sesión y volver a entrar.</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>No vuelve a abrirse solo; se puede ver con 'Ver tutorial'.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H18"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No,Parcial"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>